<commit_message>
Add JEE/NEET test type and fix analytics generation pipeline
</commit_message>
<xml_diff>
--- a/backend/uploads/generated_report.xlsx
+++ b/backend/uploads/generated_report.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Subjectwise" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2_Subjectwise'!$A$3:$M$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2_Subjectwise'!$A$3:$M$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -661,28 +661,28 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>86</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>69.67</v>
+        <v>68.33</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>83.3</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L3" s="3" t="n">
         <v>11</v>
@@ -703,102 +703,102 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>1211</t>
+          <t>1212</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Rithish S</t>
+          <t>Sanjana G S</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>44</v>
+        <v>39.33</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>65.5</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>70|75|80</t>
+          <t>60|67|73</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>1205</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Janani Sri M</t>
+          <t>Kanishk Adhithya J</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>44</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>61.1</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
@@ -813,47 +813,47 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>1201</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Kanishk Adhithya J</t>
+          <t>Adhiksha B</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>35.67</v>
+        <v>36.67</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>69.8</v>
+        <v>75</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>30</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
@@ -868,26 +868,26 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>1216</t>
+          <t>1211</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Suhana J R</t>
+          <t>Rithish S</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>107</v>
@@ -896,19 +896,19 @@
         <v>35.67</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>69.8</v>
+        <v>60.4</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
@@ -923,47 +923,47 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>1213</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Shri Vikram V</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>104</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>34.67</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="L8" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>1213</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Shri Vikram V</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>106</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>35.33</v>
-      </c>
-      <c r="I8" s="3" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>49</v>
-      </c>
-      <c r="K8" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="L8" s="3" t="n">
-        <v>18</v>
-      </c>
       <c r="M8" s="3" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -991,34 +991,34 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>30</v>
+        <v>34.33</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>56</v>
+        <v>59.6</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
@@ -1033,47 +1033,47 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>1203</t>
+          <t>1216</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Dennis Joseph A</t>
+          <t>Suhana J R</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>48</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="H10" s="3" t="n">
+        <v>34.33</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>69</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="K10" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="I10" s="3" t="n">
-        <v>52.8</v>
-      </c>
-      <c r="J10" s="3" t="n">
-        <v>53</v>
-      </c>
-      <c r="K10" s="3" t="n">
-        <v>28</v>
-      </c>
       <c r="L10" s="3" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
@@ -1088,47 +1088,47 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>1208</t>
+          <t>1214</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Pranav Barath S</t>
+          <t>Siddharth M</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>65.8</v>
+        <v>73.7</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>38</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
@@ -1143,47 +1143,47 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>1209</t>
+          <t>1219</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Pranavvi K</t>
+          <t>Harithra D</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>27.33</v>
+        <v>32.33</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>50.9</v>
+        <v>60.4</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
@@ -1198,47 +1198,47 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>1207</t>
+          <t>1209</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Kanishkhar U</t>
+          <t>Pranavvi K</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>25.67</v>
+        <v>31.33</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>49.1</v>
+        <v>56.9</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
@@ -1253,331 +1253,441 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>1212</t>
+          <t>1202</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Sanjana G S</t>
+          <t>Deekshika A G</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>24.33</v>
+        <v>30</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>51.1</v>
+        <v>65</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>48|55|62</t>
+          <t>60|67|73</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>Below Average</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>1215</t>
+          <t>1208</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Sri Asmitha R</t>
+          <t>Pranav Barath S</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="L15" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="E15" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>72</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>53.5</v>
-      </c>
-      <c r="J15" s="3" t="n">
-        <v>43</v>
-      </c>
-      <c r="K15" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="L15" s="3" t="n">
-        <v>20</v>
-      </c>
       <c r="M15" s="3" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>48|55|62</t>
+          <t>60|67|73</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>Below Average</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>1219</t>
+          <t>1203</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Harithra D</t>
+          <t>Dennis Joseph A</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>23.33</v>
+        <v>29.67</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>55</v>
+        <v>54.9</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>48|55|62</t>
+          <t>60|67|73</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>Below Average</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>1202</t>
+          <t>1205</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Deekshika A G</t>
+          <t>Janani Sri M</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="F17" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="E17" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>9</v>
-      </c>
       <c r="G17" s="3" t="n">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>21.67</v>
+        <v>29.33</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>48.9</v>
+        <v>53.8</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>48|55|62</t>
+          <t>60|67|73</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>Below Average</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>1214</t>
+          <t>1204</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Siddharth M</t>
+          <t>Gurusaran S</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>17.33</v>
+        <v>28.67</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>47.4</v>
+        <v>55.1</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>18|27|35</t>
+          <t>60|67|73</t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>1218</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Prithika R</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>83</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>27.67</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="L19" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="M19" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>60|67|73</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>1207</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Kanishkhar U</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>78</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L20" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="M20" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>60|67|73</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>1215</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Sri Asmitha R</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>19.33</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="J21" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>1201</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Adhiksha B</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>37</v>
-      </c>
-      <c r="H19" s="3" t="n">
-        <v>12.33</v>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>37.2</v>
-      </c>
-      <c r="J19" s="3" t="n">
-        <v>43</v>
-      </c>
-      <c r="K19" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="L19" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="M19" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="N19" s="3" t="inlineStr">
-        <is>
-          <t>18|27|35</t>
-        </is>
-      </c>
-      <c r="O19" s="3" t="inlineStr">
-        <is>
-          <t>Weak</t>
+      <c r="K21" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="M21" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>48|55|62</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Below Average</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1717,10 +1827,10 @@
         <v>25</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>0</v>
@@ -1730,11 +1840,11 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>84.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="K4" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
@@ -1820,27 +1930,27 @@
         </is>
       </c>
       <c r="E6" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>12</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>70.6%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="K6" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
@@ -1855,16 +1965,16 @@
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>1211</t>
+          <t>1212</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Rithish S</t>
+          <t>Sanjana G S</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -1873,27 +1983,27 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I7" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>58.3%</t>
+          <t>47.1%</t>
         </is>
       </c>
       <c r="K7" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
@@ -1902,22 +2012,22 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Needs Improvement</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>1211</t>
+          <t>1212</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Rithish S</t>
+          <t>Sanjana G S</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -1926,23 +2036,23 @@
         </is>
       </c>
       <c r="E8" s="9" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G8" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I8" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J8" s="9" t="inlineStr">
         <is>
-          <t>79.2%</t>
+          <t>76.2%</t>
         </is>
       </c>
       <c r="K8" s="9" t="n">
@@ -1961,45 +2071,45 @@
     </row>
     <row r="9">
       <c r="A9" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>1212</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Sanjana G S</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>1211</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Rithish S</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="F9" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="G9" s="10" t="n">
-        <v>5</v>
-      </c>
       <c r="H9" s="10" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>71.4%</t>
         </is>
       </c>
       <c r="K9" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
@@ -2014,49 +2124,49 @@
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>1206</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Kanishk Adhithya J</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="F10" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>1205</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Janani Sri M</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Physics</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>15</v>
-      </c>
       <c r="G10" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="H10" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="H10" s="7" t="n">
-        <v>2</v>
-      </c>
       <c r="I10" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>65.2%</t>
+          <t>58.8%</t>
         </is>
       </c>
       <c r="K10" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L10" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>7</v>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
@@ -2067,16 +2177,16 @@
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>1205</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Janani Sri M</t>
+          <t>Kanishk Adhithya J</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -2085,31 +2195,31 @@
         </is>
       </c>
       <c r="E11" s="9" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H11" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>75.0%</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>61.9%</t>
-        </is>
-      </c>
-      <c r="K11" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="L11" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -2120,16 +2230,16 @@
     </row>
     <row r="12">
       <c r="A12" s="10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>1205</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Janani Sri M</t>
+          <t>Kanishk Adhithya J</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -2141,10 +2251,10 @@
         <v>10</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H12" s="10" t="n">
         <v>15</v>
@@ -2154,15 +2264,15 @@
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="K12" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="L12" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>0</v>
+      </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="M12" s="10" t="inlineStr">
@@ -2173,16 +2283,16 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>1201</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Kanishk Adhithya J</t>
+          <t>Adhiksha B</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -2191,23 +2301,23 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>70.6%</t>
+          <t>64.3%</t>
         </is>
       </c>
       <c r="K13" s="7" t="n">
@@ -2226,16 +2336,16 @@
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>1201</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Kanishk Adhithya J</t>
+          <t>Adhiksha B</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
@@ -2244,23 +2354,23 @@
         </is>
       </c>
       <c r="E14" s="9" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G14" s="9" t="n">
         <v>3</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="9" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="K14" s="9" t="n">
@@ -2279,49 +2389,49 @@
     </row>
     <row r="15">
       <c r="A15" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>1201</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Adhiksha B</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>1206</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>Kanishk Adhithya J</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="F15" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="G15" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="H15" s="10" t="n">
-        <v>13</v>
-      </c>
       <c r="I15" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>58.3%</t>
+          <t>85.7%</t>
         </is>
       </c>
       <c r="K15" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="L15" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>2</v>
+      </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="M15" s="10" t="inlineStr">
@@ -2332,16 +2442,16 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>1216</t>
+          <t>1211</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Suhana J R</t>
+          <t>Rithish S</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -2353,10 +2463,10 @@
         <v>21</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>4</v>
@@ -2366,11 +2476,11 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>61.9%</t>
+          <t>52.4%</t>
         </is>
       </c>
       <c r="K16" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L16" s="11" t="inlineStr">
         <is>
@@ -2385,16 +2495,16 @@
     </row>
     <row r="17">
       <c r="A17" s="9" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>1216</t>
+          <t>1211</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Suhana J R</t>
+          <t>Rithish S</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -2403,23 +2513,23 @@
         </is>
       </c>
       <c r="E17" s="9" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G17" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I17" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>77.3%</t>
         </is>
       </c>
       <c r="K17" s="9" t="n">
@@ -2438,16 +2548,16 @@
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>1216</t>
+          <t>1211</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Suhana J R</t>
+          <t>Rithish S</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -2456,42 +2566,42 @@
         </is>
       </c>
       <c r="E18" s="10" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="10" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="K18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="9" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>6</v>
+      </c>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M18" s="10" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Needs Improvement</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
@@ -2509,31 +2619,31 @@
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>11</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>61.1%</t>
         </is>
       </c>
       <c r="K19" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="L19" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>7</v>
+      </c>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M19" s="7" t="inlineStr">
@@ -2544,7 +2654,7 @@
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
@@ -2562,23 +2672,23 @@
         </is>
       </c>
       <c r="E20" s="9" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="G20" s="9" t="n">
         <v>4</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>73.3%</t>
         </is>
       </c>
       <c r="K20" s="9" t="n">
@@ -2597,7 +2707,7 @@
     </row>
     <row r="21">
       <c r="A21" s="10" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
@@ -2615,42 +2725,42 @@
         </is>
       </c>
       <c r="E21" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G21" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="10" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="K21" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="L21" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>1</v>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="M21" s="10" t="inlineStr">
         <is>
-          <t>Needs Improvement</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
@@ -2668,42 +2778,42 @@
         </is>
       </c>
       <c r="E22" s="7" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I22" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>33.3%</t>
         </is>
       </c>
       <c r="K22" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="L22" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>14</v>
+      </c>
+      <c r="L22" s="12" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="M22" s="7" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>High Neg (14)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
@@ -2724,10 +2834,10 @@
         <v>16</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H23" s="9" t="n">
         <v>9</v>
@@ -2737,15 +2847,15 @@
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="K23" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="L23" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>2</v>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
@@ -2756,7 +2866,7 @@
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
@@ -2774,27 +2884,27 @@
         </is>
       </c>
       <c r="E24" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="F24" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="F24" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="G24" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="10" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="K24" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
@@ -2809,16 +2919,16 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>1203</t>
+          <t>1216</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Dennis Joseph A</t>
+          <t>Suhana J R</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -2827,51 +2937,51 @@
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I25" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>45.8%</t>
+          <t>52.9%</t>
         </is>
       </c>
       <c r="K25" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="L25" s="12" t="inlineStr">
-        <is>
-          <t>Critical</t>
+        <v>8</v>
+      </c>
+      <c r="L25" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>High Neg (13)</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>1203</t>
+          <t>1216</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Dennis Joseph A</t>
+          <t>Suhana J R</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -2880,31 +2990,31 @@
         </is>
       </c>
       <c r="E26" s="9" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G26" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="H26" s="9" t="n">
-        <v>3</v>
-      </c>
       <c r="I26" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J26" s="9" t="inlineStr">
         <is>
-          <t>63.6%</t>
+          <t>76.5%</t>
         </is>
       </c>
       <c r="K26" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="L26" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>4</v>
+      </c>
+      <c r="L26" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
@@ -2915,16 +3025,16 @@
     </row>
     <row r="27">
       <c r="A27" s="10" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>1203</t>
+          <t>1216</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Dennis Joseph A</t>
+          <t>Suhana J R</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
@@ -2933,51 +3043,51 @@
         </is>
       </c>
       <c r="E27" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F27" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="F27" s="10" t="n">
-        <v>3</v>
-      </c>
       <c r="G27" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J27" s="10" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="K27" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="L27" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>1</v>
+      </c>
+      <c r="L27" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="M27" s="10" t="inlineStr">
         <is>
-          <t>Needs Improvement</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>1208</t>
+          <t>1214</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Pranav Barath S</t>
+          <t>Siddharth M</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -2986,27 +3096,27 @@
         </is>
       </c>
       <c r="E28" s="7" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F28" s="7" t="n">
         <v>7</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H28" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I28" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>53.8%</t>
         </is>
       </c>
       <c r="K28" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
@@ -3021,16 +3131,16 @@
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>1208</t>
+          <t>1214</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Pranav Barath S</t>
+          <t>Siddharth M</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
@@ -3042,10 +3152,10 @@
         <v>14</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H29" s="9" t="n">
         <v>11</v>
@@ -3055,11 +3165,11 @@
       </c>
       <c r="J29" s="9" t="inlineStr">
         <is>
-          <t>85.7%</t>
+          <t>78.6%</t>
         </is>
       </c>
       <c r="K29" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
@@ -3074,16 +3184,16 @@
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>1208</t>
+          <t>1214</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Pranav Barath S</t>
+          <t>Siddharth M</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
@@ -3092,31 +3202,31 @@
         </is>
       </c>
       <c r="E30" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F30" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="F30" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="G30" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J30" s="10" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>90.9%</t>
         </is>
       </c>
       <c r="K30" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="L30" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>1</v>
+      </c>
+      <c r="L30" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="M30" s="10" t="inlineStr">
@@ -3127,16 +3237,16 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>1209</t>
+          <t>1219</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Pranavvi K</t>
+          <t>Harithra D</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -3145,51 +3255,51 @@
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>28.6%</t>
+          <t>38.9%</t>
         </is>
       </c>
       <c r="K31" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="L31" s="12" t="inlineStr">
-        <is>
-          <t>Critical</t>
+        <v>11</v>
+      </c>
+      <c r="L31" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>High Neg (15)</t>
+          <t>Needs Improvement</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>1209</t>
+          <t>1219</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Pranavvi K</t>
+          <t>Harithra D</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
@@ -3201,10 +3311,10 @@
         <v>20</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H32" s="9" t="n">
         <v>5</v>
@@ -3214,11 +3324,11 @@
       </c>
       <c r="J32" s="9" t="inlineStr">
         <is>
-          <t>65.0%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="K32" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
@@ -3233,16 +3343,16 @@
     </row>
     <row r="33">
       <c r="A33" s="10" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>1209</t>
+          <t>1219</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Pranavvi K</t>
+          <t>Harithra D</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
@@ -3251,31 +3361,31 @@
         </is>
       </c>
       <c r="E33" s="10" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F33" s="10" t="n">
         <v>8</v>
       </c>
       <c r="G33" s="10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J33" s="10" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="K33" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="L33" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>2</v>
+      </c>
+      <c r="L33" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="M33" s="10" t="inlineStr">
@@ -3286,16 +3396,16 @@
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>1207</t>
+          <t>1209</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Kanishkhar U</t>
+          <t>Pranavvi K</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -3304,27 +3414,27 @@
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F34" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H34" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I34" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>52.9%</t>
         </is>
       </c>
       <c r="K34" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L34" s="11" t="inlineStr">
         <is>
@@ -3339,16 +3449,16 @@
     </row>
     <row r="35">
       <c r="A35" s="9" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>1207</t>
+          <t>1209</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Kanishkhar U</t>
+          <t>Pranavvi K</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
@@ -3357,23 +3467,23 @@
         </is>
       </c>
       <c r="E35" s="9" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G35" s="9" t="n">
         <v>9</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I35" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J35" s="9" t="inlineStr">
         <is>
-          <t>52.6%</t>
+          <t>59.1%</t>
         </is>
       </c>
       <c r="K35" s="9" t="n">
@@ -3392,16 +3502,16 @@
     </row>
     <row r="36">
       <c r="A36" s="10" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>1207</t>
+          <t>1209</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Kanishkhar U</t>
+          <t>Pranavvi K</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
@@ -3410,51 +3520,51 @@
         </is>
       </c>
       <c r="E36" s="10" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F36" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G36" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="G36" s="10" t="n">
-        <v>9</v>
-      </c>
       <c r="H36" s="10" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J36" s="10" t="inlineStr">
         <is>
-          <t>35.7%</t>
+          <t>58.3%</t>
         </is>
       </c>
       <c r="K36" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="L36" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>5</v>
+      </c>
+      <c r="L36" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M36" s="10" t="inlineStr">
         <is>
-          <t>Needs Improvement</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>1212</t>
+          <t>1202</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Sanjana G S</t>
+          <t>Deekshika A G</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -3463,51 +3573,51 @@
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="I37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>64.3%</t>
         </is>
       </c>
       <c r="K37" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="L37" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>5</v>
+      </c>
+      <c r="L37" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>Needs Improvement</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>1212</t>
+          <t>1202</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Sanjana G S</t>
+          <t>Deekshika A G</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
@@ -3516,27 +3626,27 @@
         </is>
       </c>
       <c r="E38" s="9" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F38" s="9" t="n">
         <v>8</v>
       </c>
       <c r="G38" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I38" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J38" s="9" t="inlineStr">
         <is>
-          <t>53.3%</t>
+          <t>61.5%</t>
         </is>
       </c>
       <c r="K38" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L38" s="8" t="inlineStr">
         <is>
@@ -3551,16 +3661,16 @@
     </row>
     <row r="39">
       <c r="A39" s="10" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>1212</t>
+          <t>1202</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Sanjana G S</t>
+          <t>Deekshika A G</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
@@ -3569,23 +3679,23 @@
         </is>
       </c>
       <c r="E39" s="10" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G39" s="10" t="n">
         <v>4</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J39" s="10" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>69.2%</t>
         </is>
       </c>
       <c r="K39" s="10" t="n">
@@ -3604,16 +3714,16 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>1215</t>
+          <t>1208</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Sri Asmitha R</t>
+          <t>Pranav Barath S</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
@@ -3622,23 +3732,23 @@
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G40" s="7" t="n">
         <v>10</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I40" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>41.2%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="K40" s="7" t="n">
@@ -3657,16 +3767,16 @@
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>1215</t>
+          <t>1208</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Sri Asmitha R</t>
+          <t>Pranav Barath S</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -3675,31 +3785,31 @@
         </is>
       </c>
       <c r="E41" s="9" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H41" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I41" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="9" t="inlineStr">
+        <is>
+          <t>73.7%</t>
+        </is>
+      </c>
+      <c r="K41" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="I41" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" s="9" t="inlineStr">
-        <is>
-          <t>60.0%</t>
-        </is>
-      </c>
-      <c r="K41" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="L41" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="L41" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M41" s="9" t="inlineStr">
@@ -3710,16 +3820,16 @@
     </row>
     <row r="42">
       <c r="A42" s="10" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>1215</t>
+          <t>1208</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>Sri Asmitha R</t>
+          <t>Pranav Barath S</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
@@ -3728,27 +3838,27 @@
         </is>
       </c>
       <c r="E42" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F42" s="10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G42" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H42" s="10" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="I42" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J42" s="10" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="K42" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L42" s="9" t="inlineStr">
         <is>
@@ -3763,16 +3873,16 @@
     </row>
     <row r="43">
       <c r="A43" s="7" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>1219</t>
+          <t>1203</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Harithra D</t>
+          <t>Dennis Joseph A</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -3784,10 +3894,10 @@
         <v>20</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G43" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H43" s="7" t="n">
         <v>5</v>
@@ -3797,11 +3907,11 @@
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="K43" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L43" s="11" t="inlineStr">
         <is>
@@ -3816,16 +3926,16 @@
     </row>
     <row r="44">
       <c r="A44" s="9" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>1219</t>
+          <t>1203</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Harithra D</t>
+          <t>Dennis Joseph A</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
@@ -3834,27 +3944,27 @@
         </is>
       </c>
       <c r="E44" s="9" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="G44" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I44" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J44" s="9" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>60.9%</t>
         </is>
       </c>
       <c r="K44" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L44" s="11" t="inlineStr">
         <is>
@@ -3863,22 +3973,22 @@
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>Needs Improvement</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>1219</t>
+          <t>1203</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>Harithra D</t>
+          <t>Dennis Joseph A</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
@@ -3887,31 +3997,31 @@
         </is>
       </c>
       <c r="E45" s="10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F45" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G45" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="K45" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="L45" s="9" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>4</v>
+      </c>
+      <c r="L45" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M45" s="10" t="inlineStr">
@@ -3922,16 +4032,16 @@
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>1202</t>
+          <t>1205</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Deekshika A G</t>
+          <t>Janani Sri M</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -3943,10 +4053,10 @@
         <v>19</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H46" s="7" t="n">
         <v>6</v>
@@ -3956,11 +4066,11 @@
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>36.8%</t>
+          <t>42.1%</t>
         </is>
       </c>
       <c r="K46" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L46" s="11" t="inlineStr">
         <is>
@@ -3975,16 +4085,16 @@
     </row>
     <row r="47">
       <c r="A47" s="9" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>1202</t>
+          <t>1205</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Deekshika A G</t>
+          <t>Janani Sri M</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
@@ -3993,31 +4103,31 @@
         </is>
       </c>
       <c r="E47" s="9" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F47" s="9" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H47" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I47" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="9" t="inlineStr">
+        <is>
+          <t>73.7%</t>
+        </is>
+      </c>
+      <c r="K47" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="I47" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" s="9" t="inlineStr">
-        <is>
-          <t>60.0%</t>
-        </is>
-      </c>
-      <c r="K47" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="L47" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="L47" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M47" s="9" t="inlineStr">
@@ -4028,16 +4138,16 @@
     </row>
     <row r="48">
       <c r="A48" s="10" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>1202</t>
+          <t>1205</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>Deekshika A G</t>
+          <t>Janani Sri M</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
@@ -4046,51 +4156,51 @@
         </is>
       </c>
       <c r="E48" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="F48" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="F48" s="10" t="n">
-        <v>3</v>
-      </c>
       <c r="G48" s="10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H48" s="10" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J48" s="10" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="K48" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="L48" s="9" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>8</v>
+      </c>
+      <c r="L48" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="M48" s="10" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Needs Improvement</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>1214</t>
+          <t>1204</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Siddharth M</t>
+          <t>Gurusaran S</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -4099,27 +4209,27 @@
         </is>
       </c>
       <c r="E49" s="7" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G49" s="7" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I49" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>42.1%</t>
         </is>
       </c>
       <c r="K49" s="7" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="L49" s="11" t="inlineStr">
         <is>
@@ -4134,16 +4244,16 @@
     </row>
     <row r="50">
       <c r="A50" s="9" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>1214</t>
+          <t>1204</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Siddharth M</t>
+          <t>Gurusaran S</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
@@ -4152,27 +4262,27 @@
         </is>
       </c>
       <c r="E50" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="G50" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H50" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="F50" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="G50" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="H50" s="9" t="n">
-        <v>17</v>
-      </c>
       <c r="I50" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J50" s="9" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>58.8%</t>
         </is>
       </c>
       <c r="K50" s="9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L50" s="8" t="inlineStr">
         <is>
@@ -4187,16 +4297,16 @@
     </row>
     <row r="51">
       <c r="A51" s="10" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>1214</t>
+          <t>1204</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>Siddharth M</t>
+          <t>Gurusaran S</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
@@ -4205,51 +4315,51 @@
         </is>
       </c>
       <c r="E51" s="10" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F51" s="10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G51" s="10" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H51" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J51" s="10" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>69.2%</t>
         </is>
       </c>
       <c r="K51" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="L51" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>4</v>
+      </c>
+      <c r="L51" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M51" s="10" t="inlineStr">
         <is>
-          <t>Needs Improvement</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>1201</t>
+          <t>1218</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Adhiksha B</t>
+          <t>Prithika R</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -4258,51 +4368,51 @@
         </is>
       </c>
       <c r="E52" s="7" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G52" s="7" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H52" s="7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>52.9%</t>
         </is>
       </c>
       <c r="K52" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="L52" s="12" t="inlineStr">
-        <is>
-          <t>Critical</t>
+        <v>8</v>
+      </c>
+      <c r="L52" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="M52" s="7" t="inlineStr">
         <is>
-          <t>High Neg (14)</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>1201</t>
+          <t>1218</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Adhiksha B</t>
+          <t>Prithika R</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
@@ -4311,51 +4421,51 @@
         </is>
       </c>
       <c r="E53" s="9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F53" s="9" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G53" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H53" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="H53" s="9" t="n">
-        <v>10</v>
-      </c>
       <c r="I53" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J53" s="9" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>68.8%</t>
         </is>
       </c>
       <c r="K53" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="L53" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>5</v>
+      </c>
+      <c r="L53" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M53" s="9" t="inlineStr">
         <is>
-          <t>Needs Improvement</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>1201</t>
+          <t>1218</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>Adhiksha B</t>
+          <t>Prithika R</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
@@ -4364,23 +4474,23 @@
         </is>
       </c>
       <c r="E54" s="10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F54" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G54" s="10" t="n">
         <v>4</v>
       </c>
       <c r="H54" s="10" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J54" s="10" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="K54" s="10" t="n">
@@ -4393,12 +4503,330 @@
       </c>
       <c r="M54" s="10" t="inlineStr">
         <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>1207</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Kanishkhar U</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="F55" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="G55" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H55" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="I55" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="7" t="inlineStr">
+        <is>
+          <t>44.4%</t>
+        </is>
+      </c>
+      <c r="K55" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="L55" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M55" s="7" t="inlineStr">
+        <is>
           <t>Needs Improvement</t>
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>1207</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>Kanishkhar U</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="F56" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="G56" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H56" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="I56" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="9" t="inlineStr">
+        <is>
+          <t>47.1%</t>
+        </is>
+      </c>
+      <c r="K56" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="L56" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>Needs Improvement</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>1207</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>Kanishkhar U</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="F57" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G57" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="H57" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I57" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="10" t="inlineStr">
+        <is>
+          <t>58.8%</t>
+        </is>
+      </c>
+      <c r="K57" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L57" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="M57" s="10" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>1215</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Sri Asmitha R</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="F58" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G58" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H58" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="I58" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>38.5%</t>
+        </is>
+      </c>
+      <c r="K58" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L58" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t>Needs Improvement</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>1215</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>Sri Asmitha R</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="F59" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="G59" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H59" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="I59" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="9" t="inlineStr">
+        <is>
+          <t>69.2%</t>
+        </is>
+      </c>
+      <c r="K59" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L59" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="M59" s="9" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>1215</t>
+        </is>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>Sri Asmitha R</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E60" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F60" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G60" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="H60" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="I60" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" s="10" t="inlineStr">
+        <is>
+          <t>45.5%</t>
+        </is>
+      </c>
+      <c r="K60" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L60" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="M60" s="10" t="inlineStr">
+        <is>
+          <t>Needs Improvement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:M54"/>
+  <autoFilter ref="A3:M60"/>
   <mergeCells count="2">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>

</xml_diff>